<commit_message>
chore(abdm-ft): mask patient details in the M2 test artifacts
- Dates and years of birth masked in the tracked M2 text files and both
  M2 workbooks, archive included.
- Names, initials and dates of birth masked in the 17 current screenshots
  that showed them, and the report rebuilt from them as version 1.2.

The 30 archived screenshots, and the two archived reports that embed
them, are not masked yet. Earlier commits still hold the unmasked files.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/abdm-ft/archive/final-20261029-before-share-rerun/M2_BUILDING_HIP_TEST_CASES.xlsx
+++ b/abdm-ft/archive/final-20261029-before-share-rerun/M2_BUILDING_HIP_TEST_CASES.xlsx
@@ -1553,7 +1553,7 @@
       <c r="J19" s="14" t="n"/>
       <c r="K19" s="14" t="inlineStr">
         <is>
-          <t>Inbound POST /api/v3/hip/patient/care-context/discover REQUEST-ID 17df06aa-b95d-4f33-b2d0-5ba9cbf0677b at 23:24:10 IST: transactionId f3c99f71-3824-4f30-8a2b-afc473b1f443 present, patient.id present, patient.verifiedIdentifiers [MOBILE, ABHA_NUMBER, abhaAddress], gender F, yearOfBirth 2004</t>
+          <t>Inbound POST /api/v3/hip/patient/care-context/discover REQUEST-ID 17df06aa-b95d-4f33-b2d0-5ba9cbf0677b at 23:24:10 IST: transactionId f3c99f71-3824-4f30-8a2b-afc473b1f443 present, patient.id present, patient.verifiedIdentifiers [MOBILE, ABHA_NUMBER, abhaAddress], gender F, yearOfBirth [masked]</t>
         </is>
       </c>
       <c r="L19" s="14" t="inlineStr">
@@ -1610,7 +1610,7 @@
       <c r="J20" s="16" t="n"/>
       <c r="K20" s="16" t="inlineStr">
         <is>
-          <t>Matched by MOBILE to patient OCM123-2026-0013 (registered without ABHA; Female, born 2004, mobile ending 5506); on-discover sent with matchedBy [MOBILE] and patient[].careContexts [RX-67209C38-D094-4EB0-B928-A13D4529CF57], accepted by ABDM; the PHR app showed that record under our patient reference (USER_INIT_LINK_604/phr-1.png)</t>
+          <t>Matched by MOBILE to patient OCM123-2026-0013 (registered without ABHA; Female, born [masked], mobile ending 5506); on-discover sent with matchedBy [MOBILE] and patient[].careContexts [RX-67209C38-D094-4EB0-B928-A13D4529CF57], accepted by ABDM; the PHR app showed that record under our patient reference (USER_INIT_LINK_604/phr-1.png)</t>
         </is>
       </c>
       <c r="L20" s="16" t="inlineStr">
@@ -1623,7 +1623,7 @@
       </c>
       <c r="N20" s="16" t="inlineStr">
         <is>
-          <t>Screen check: the matched patient's mobile, gender (F) and year of birth (2004) agree with the discover's. The build does not store outbound reply bodies: the on-discover content is shown by the PHR screen and by the init that selected from it.</t>
+          <t>Screen check: the matched patient's mobile, gender (F) and year of birth ([masked]) agree with the discover's. The build does not store outbound reply bodies: the on-discover content is shown by the PHR screen and by the init that selected from it.</t>
         </is>
       </c>
       <c r="O20" s="55" t="n"/>

</xml_diff>